<commit_message>
Fix: Route handler types and async params for Next.js 16
</commit_message>
<xml_diff>
--- a/storage/Accounting_Ledger.xlsx
+++ b/storage/Accounting_Ledger.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="10">
   <si>
     <t>TANGGAL</t>
   </si>
@@ -35,6 +35,12 @@
   </si>
   <si>
     <t>Import Invoice Invoice</t>
+  </si>
+  <si>
+    <t>0001/INV-FDL/I/2026</t>
+  </si>
+  <si>
+    <t>PT. Mercury Tekindo Internusa</t>
   </si>
 </sst>
 </file>
@@ -45,7 +51,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="_(&quot;Rp&quot;* #,##0_);_(&quot;Rp&quot;* (#,##0);_(&quot;Rp&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -57,6 +63,9 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -91,7 +100,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -100,6 +109,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -440,7 +464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -530,6 +554,26 @@
         <v>1045000</v>
       </c>
     </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="5">
+        <v>46052</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="8">
+        <v>44500000</v>
+      </c>
+      <c r="E5" s="8">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9">
+        <v>45545000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>